<commit_message>
feat: complete portable AI quality orchestration workflow
</commit_message>
<xml_diff>
--- a/requirements/salary-trade/outputs/structured-test-cases.xlsx
+++ b/requirements/salary-trade/outputs/structured-test-cases.xlsx
@@ -294,7 +294,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -371,7 +371,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -3220,7 +3220,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -3990,7 +3990,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -4144,7 +4144,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -5838,7 +5838,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -5915,7 +5915,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -5992,7 +5992,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -6069,7 +6069,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -6146,7 +6146,7 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
@@ -6223,7 +6223,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -6300,7 +6300,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -6377,7 +6377,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -6531,7 +6531,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
@@ -6685,7 +6685,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -6839,7 +6839,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -6916,7 +6916,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -6993,7 +6993,7 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -7070,7 +7070,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -7147,7 +7147,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -7224,7 +7224,7 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -7301,7 +7301,7 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -7378,7 +7378,7 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -7532,7 +7532,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -7917,7 +7917,7 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -8841,7 +8841,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -8918,7 +8918,7 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -8995,7 +8995,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -10689,7 +10689,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
@@ -10766,7 +10766,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -10843,7 +10843,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -10920,7 +10920,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -10997,7 +10997,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -11074,7 +11074,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
@@ -11151,7 +11151,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L145" t="inlineStr">
@@ -11228,7 +11228,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
@@ -11305,7 +11305,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L147" t="inlineStr">
@@ -11382,7 +11382,7 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L148" t="inlineStr">
@@ -11459,7 +11459,7 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L150" t="inlineStr">
@@ -11613,7 +11613,7 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L151" t="inlineStr">
@@ -11690,7 +11690,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L152" t="inlineStr">
@@ -11767,7 +11767,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
@@ -11844,7 +11844,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L154" t="inlineStr">
@@ -11921,7 +11921,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L155" t="inlineStr">
@@ -11998,7 +11998,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L156" t="inlineStr">
@@ -12075,7 +12075,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L157" t="inlineStr">
@@ -12152,7 +12152,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L158" t="inlineStr">
@@ -12229,7 +12229,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L159" t="inlineStr">
@@ -12306,7 +12306,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L160" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>country_code, currency, proxy_uid</t>
+          <t>currency, proxy_uid</t>
         </is>
       </c>
       <c r="L161" t="inlineStr">

</xml_diff>